<commit_message>
Translate the repository into English: file names, documents, workbooks, registers, logs, code messages and web interface; passage text removed from review workbooks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/eval/dev_questions.xlsx
+++ b/data/eval/dev_questions.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选项" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="专题" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,63 +448,63 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>苹果病虫害 RAG 题库模板（每题一行，填写“questions”页）</t>
+          <t>Apple pest and disease RAG question bank template (one question per row, fill in the "questions" sheet)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. 先在原文中定位事实，再写问题和参考答案；不要先问模型再把模型答案当参考答案。</t>
+          <t>1. Locate the facts in the source first, then write the question and reference answer; never use a model answer as the reference answer.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. 每题 3–5 个必答要点，评分 0–4 分对照这些要点。</t>
+          <t>2. Each question has 3–5 required points; the 0–4 score is given against these points.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. chunk_ids 填数据库片段 ID（可在问答页证据卡或 web_chunks_reviewed.json 查找）；check 命令会核对其存在。</t>
+          <t>3. chunk_ids are database chunk IDs (see the evidence cards in the Q&amp;A page or web_chunks_reviewed.json); the check command verifies that they exist.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. 开发集与测试集按专题和问题类型分开，不要把同一问题改写后放进两组。</t>
+          <t>4. Keep the development and test sets apart by topic and question type; never put a rewritten version of the same question in both.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5. 参考答案须由另一名成员复核，复核通过后 status 改为 reviewed。冻结前运行：python 代码/tools/question_bank.py check 文件.xlsx --export</t>
+          <t>5. Another member must review each reference answer; after review set status to reviewed. Before freezing run: python code/tools/question_bank.py check FILE.xlsx --export</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6. 被测系统只能收到 question_en；参考答案和评分标准不得进入提示词。</t>
+          <t>6. The tested system receives only question_en; reference answers and scoring criteria never enter the prompt.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7. 示例行 D001、D002 正式填写前删除。</t>
+          <t>7. Delete example rows D001 and D002 before use.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>计划配额（测试集 60 题，开发集 20 题按同样类型分布）：</t>
+          <t>Planned quota (test set 60 questions; development set 20 questions with the same distribution):</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>D001–D020 开发集；T001–T060 测试集，唯一且不复用</t>
+          <t>D001–D020 development set; T001–T060 test set; unique and never reused</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -701,77 +701,77 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>范围表编号 T01–T46，见“专题”页</t>
+          <t>Scope table identifier T01–T46, see the "Topics" sheet</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>见“选项”页</t>
+          <t>See the "Options" sheet</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>证据所属地区，如 United States - Pacific Northwest / New Zealand</t>
+          <t>Region of the evidence, e.g. United States - Pacific Northwest / New Zealand</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>生育/采后阶段</t>
+          <t>Growth or postharvest stage</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>answerable / partial / unanswerable（语料内）</t>
+          <t>answerable / partial / unanswerable (within the corpus)</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>英文问题；写明地区或来源情境，不出现答案线索</t>
+          <t>Question in English; state region or source context; no answer hints</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>只依据所引原文写成的参考答案</t>
+          <t>Reference answer written only from the cited passages</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>3–5 个必答要点，用 | 分隔；评分 0–4 依据</t>
+          <t>3–5 required points separated by |; basis for the 0–4 score</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>判为重大错误的情形，用 | 分隔</t>
+          <t>Cases counted as major errors, separated by |</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>边界题：可答部分 / 应拒答部分 / 理由</t>
+          <t>Boundary questions: answerable part / part to decline / reason</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>如 S001|S036</t>
+          <t>e.g. S001|S036</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>如 S001:web:3|S001:web:4（可用多个等价片段）</t>
+          <t>e.g. S001:web:3|S001:web:4 (several equivalent chunks allowed)</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>PDF 页码或网页章节，如 p.12 / Symptoms and Signs</t>
+          <t>PDF page or web section, e.g. p.12 / Symptoms and Signs</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>出题人</t>
+          <t>Author</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>复核人，必须不同于出题人</t>
+          <t>Reviewer; must differ from the author</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
@@ -781,12 +781,12 @@
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>从 1 开始，修改后加 1</t>
+          <t>Starts at 1; add 1 after each change</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>争议、地区转用、来源冲突等</t>
+          <t>Disputes, regional transfer, source conflicts, etc.</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Review 2026-10-16 [missing citation]: Claim that rust mites need a hand lens was supported only by an uncited chunk.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Review 2026-10-16 [missing citation]: Claim that rust mites need a hand lens was supported only by an uncited chunk.</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="T6" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; S089 原始发表于 1993; Review 2026-10-16 [beyond source]: "with larvae inside" is not stated in S087:9; source says midge larvae feed along leaf margins.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; S089 originally published in 1993; Review 2026-10-16 [beyond source]: "with larvae inside" is not stated in S087:9; source says midge larvae feed along leaf margins.</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Review 2026-10-16 [wording]: Source mentions galleries, not "beetle holes".</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Review 2026-10-16 [wording]: Source mentions galleries, not "beetle holes".</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; 提问未说明地区；参考答案给出新西兰 S265 的具体修剪长度并注明来源; Review 2026-10-16 [missing key differentiator]: S066 states bacterial ooze is never present with blossom blast; "Gala is highly susceptible" overstated the UC IPM wording.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; region not stated in the question; the reference answer gives the specific pruning length from New Zealand source S265 and names the source; Review 2026-10-16 [missing key differentiator]: S066 states bacterial ooze is never present with blossom blast; "Gala is highly susceptible" overstated the UC IPM wording.</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Review 2026-10-16 [beyond source]: "reduce root infestation" is an inference; S020:6 says the rootstocks were developed to be resistant.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Review 2026-10-16 [beyond source]: "reduce root infestation" is an inference; S020:6 says the rootstocks were developed to be resistant.</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>农户口吻 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>Farmer's voice v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>附带地区/环境 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Review 2026-10-16 [editing error]: WSU sentence was duplicated at the end; the WSU spray recommendation is conditional on the orchard being threatened.</t>
+          <t>With region or environment context v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Review 2026-10-16 [editing error]: WSU sentence was duplicated at the end; the WSU spray recommendation is conditional on the orchard being threatened.</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>附带地区/环境 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>With region or environment context v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>附带地区/环境 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Review 2026-10-16 [wording]: S074:11 says to position bins to minimise soil contamination of their undersides, not to keep bins off the soil.</t>
+          <t>With region or environment context v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Review 2026-10-16 [wording]: S074:11 says to position bins to minimise soil contamination of their undersides, not to keep bins off the soil.</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>可答：可能原因、新西兰土壤翻耕试验；应拒答：药剂与施药时机；理由：语料无新西兰化学防治依据</t>
+          <t>Answerable: likely cause, New Zealand soil cultivation trial; decline: products and spray timing; reason: the corpus has no New Zealand chemical control evidence</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>附带地区/环境 v2; 提问者自述在新西兰; Review 2026-10-16 [beyond source]: "checking at night to see the beetles would confirm it" is not in the source.</t>
+          <t>With region or environment context v2; asker states they are in New Zealand; Review 2026-10-16 [beyond source]: "checking at night to see the beetles would confirm it" is not in the source.</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>可答：感染时期、海外果园措施；应拒答：新西兰储藏温度；理由：语料无此依据</t>
+          <t>Answerable: infection period, overseas orchard measures; decline: New Zealand storage temperature; reason: no such evidence in the corpus</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>附带地区/环境 v2; 提问者自述在新西兰; Review 2026-10-16 [beyond source]: "storage temperature is not the main control" is an inference not stated by any source.</t>
+          <t>With region or environment context v2; asker states they are in New Zealand; Review 2026-10-16 [beyond source]: "storage temperature is not the main control" is an inference not stated by any source.</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2488,7 @@
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>可答：海外抗性砧木及其不确定性；应限定：非新西兰验证；理由：语料无新西兰砧木试验</t>
+          <t>Answerable: overseas resistant rootstocks and their uncertainty; qualify: not validated in New Zealand; reason: the corpus has no New Zealand rootstock trial</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>附带地区/环境 v2; 提问者自述在新西兰; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
+          <t>With region or environment context v2; asker states they are in New Zealand; Evidence check: every statement and number traced to cited chunks; no change needed.</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2622,7 @@
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>偏僻专题 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Review 2026-10-16 [substantive error]: Yellowing and early leaf drop were given as a differentiator, but S174 states apple scab also causes leaves to yellow and drop prematurely.</t>
+          <t>Rare topic v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Review 2026-10-16 [substantive error]: Yellowing and early leaf drop were given as a differentiator, but S174 states apple scab also causes leaves to yellow and drop prematurely.</t>
         </is>
       </c>
     </row>
@@ -2718,26 +2718,26 @@
       </c>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>偏僻专题 v2; 提问者未说明地区；评分接受任何有依据的来源，但地区性数值须注明来源地区; Review 2026-10-16 [substantive error]: Penn State spray timing (from pink bud) is written for cedar-apple rust; quince rust infection window starts at tight cluster, so it was misattributed.</t>
+          <t>Rare topic v2; region not stated by the asker; any supported source is accepted in scoring, but regional values must state their source region; Review 2026-10-16 [substantive error]: Penn State spray timing (from pink bud) is written for cedar-apple rust; quince rust infection window starts at tight cluster, so it was misattributed.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='选项'!$A$2:$A$3</formula1>
+      <formula1>='Options'!$A$2:$A$3</formula1>
     </dataValidation>
     <dataValidation sqref="D3:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='选项'!$B$2:$B$7</formula1>
+      <formula1>='Options'!$B$2:$B$7</formula1>
     </dataValidation>
     <dataValidation sqref="G3:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='选项'!$C$2:$C$4</formula1>
+      <formula1>='Options'!$C$2:$C$4</formula1>
     </dataValidation>
     <dataValidation sqref="F3:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='选项'!$D$2:$D$7</formula1>
+      <formula1>='Options'!$D$2:$D$7</formula1>
     </dataValidation>
     <dataValidation sqref="R3:R500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='选项'!$E$2:$E$5</formula1>
+      <formula1>='Options'!$E$2:$E$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Apple scab 苹果黑星病</t>
+          <t>Apple scab</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fire blight 火疫病</t>
+          <t>Fire blight</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Powdery mildew 白粉病</t>
+          <t>Powdery mildew</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>European canker 欧洲溃疡病</t>
+          <t>European canker</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Apple anthracnose 苹果炭疽溃疡类专题</t>
+          <t>Apple anthracnose (canker) topic</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Phytophthora root/crown rot 疫霉根腐病</t>
+          <t>Phytophthora root/crown rot</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Armillaria root rot 蜜环菌根腐病</t>
+          <t>Armillaria root rot</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bacterial blossom blast 细菌性花枯</t>
+          <t>Bacterial blossom blast</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Black rot / Frogeye leaf spot 黑腐病</t>
+          <t>Black rot / Frogeye leaf spot</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3145,7 +3145,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bitter rot 苦腐病</t>
+          <t>Bitter rot</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>White rot 白腐病</t>
+          <t>White rot</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sooty blotch / Flyspeck 煤污病与蝇粪病</t>
+          <t>Sooty blotch / Flyspeck</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cedar apple / Quince rust 锈病</t>
+          <t>Cedar apple / Quince rust</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Blue mold 青霉病</t>
+          <t>Blue mold</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gray mold 灰霉病</t>
+          <t>Gray mold</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bull's eye rot 牛眼腐病</t>
+          <t>Bull's eye rot</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mucor rot 毛霉腐烂</t>
+          <t>Mucor rot</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Marssonina blotch 苹果褐斑病</t>
+          <t>Marssonina blotch</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Crown gall 根癌病</t>
+          <t>Crown gall</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Core rot / Moldy core 果心腐烂</t>
+          <t>Core rot / Moldy core</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Apple replant disease 连作障碍专题</t>
+          <t>Apple replant disease topic</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Codling moth 苹果蠹蛾</t>
+          <t>Codling moth</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Apple maggot 苹果实蝇</t>
+          <t>Apple maggot</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Woolly apple aphid 苹果绵蚜</t>
+          <t>Woolly apple aphid</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Green/apple/spirea aphids 苹果蚜类</t>
+          <t>Green/apple/spirea aphids</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Leafrollers 卷叶蛾类</t>
+          <t>Leafrollers</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Lightbrown apple moth 浅褐苹果蛾</t>
+          <t>Lightbrown apple moth</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>European red mite 欧洲红蜘蛛</t>
+          <t>European red mite</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Spider mites 叶螨类</t>
+          <t>Spider mites</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Apple rust mite 苹果锈螨</t>
+          <t>Apple rust mite</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>San Jose scale 圣何塞蚧</t>
+          <t>San Jose scale</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Leafminers 潜叶蛾类</t>
+          <t>Leafminers</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Leafhoppers 叶蝉类</t>
+          <t>Leafhoppers</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Brown marmorated stink bug 褐斑蝽</t>
+          <t>Brown marmorated stink bug</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Bronze beetle 铜色甲虫</t>
+          <t>Bronze beetle</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Oriental fruit moth 东方果蛾</t>
+          <t>Oriental fruit moth</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Plum curculio 李象甲</t>
+          <t>Plum curculio</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Apple mosaic 苹果花叶病</t>
+          <t>Apple mosaic</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Apple leafcurling midge 苹果卷叶瘿蚊</t>
+          <t>Apple leafcurling midge</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3878,7 +3878,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Mealybugs 粉蚧类（苹果）</t>
+          <t>Mealybugs (apple)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alternaria 相关苹果病害</t>
+          <t>Alternaria-related apple diseases</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Elsinoe 相关苹果病害</t>
+          <t>Elsinoe-related apple diseases</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">

</xml_diff>